<commit_message>
Akro-Mils re-layout from bin spreadsheet; merge Elastic Band Anchor Plate
- Apply Gavin's Akro-Mils drawer assignments (AK01-AK42), with drawer labels
- Rubber Shaft Collar, 2x and 6x Pitch Standoff now span two drawers
- Merge EES "Elastic Band Anchor Plate" (228-3616-157) into Rubber Band
  Anchor: same part in a different color; qty 41, B3-8
- Regenerate bin-assignments.xlsx and images/sizes.json (162 parts)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/bin-assignments.xlsx
+++ b/tools/bin-assignments.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bins'!$A$1:$H$179</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parts'!$A$1:$E$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parts'!$A$1:$E$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2793,12 +2793,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Elastic Band Anchor Plate</t>
+          <t>Shaft Bushing</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Elastic Band Anchor Plate</t>
+          <t>Shaft Bushing</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,16 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Washers</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Washer</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
@@ -2828,12 +2837,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Washers</t>
+          <t>0.25x Spacer</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Washer</t>
+          <t>0.25x Pitch Spacer</t>
         </is>
       </c>
     </row>
@@ -2850,12 +2859,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Rubber Shaft Collars</t>
+          <t>0.5x Spacer</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Rubber Shaft Collar</t>
+          <t>0.5x Pitch Spacer</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2892,16 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Rubber Shaft Collars</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Rubber Shaft Collar</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
@@ -2896,7 +2914,16 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Rubber Shaft Collars</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Rubber Shaft Collar</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
@@ -2974,16 +3001,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>1x Plastic Motor Shaft</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>1x Pitch Plastic Motor Shaft</t>
-        </is>
-      </c>
+      <c r="C108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
@@ -2996,16 +3014,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>2x Plastic Motor Shaft</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>2x Pitch Plastic Motor Shaft</t>
-        </is>
-      </c>
+      <c r="C109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
@@ -3018,16 +3027,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>3x Plastic Motor Shaft</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>3x Pitch Plastic Motor Shaft</t>
-        </is>
-      </c>
+      <c r="C110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
@@ -3040,16 +3040,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>4x Plastic Motor Shaft</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>4x Pitch Plastic Motor Shaft</t>
-        </is>
-      </c>
+      <c r="C111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
@@ -3064,12 +3055,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>3x Capped Plastic Shaft</t>
+          <t>2x Capped Shaft</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>3x Pitch Capped Plastic Shaft</t>
+          <t>2x Pitch Capped Shaft</t>
         </is>
       </c>
     </row>
@@ -3086,12 +3077,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>5x Capped Plastic Shaft</t>
+          <t>3x Capped Shafts (plastic + metal)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>5x Pitch Capped Plastic Shaft</t>
+          <t>3x Pitch Capped Plastic Shaft</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>3x Pitch Capped Shaft</t>
         </is>
       </c>
     </row>
@@ -3108,12 +3104,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2x Capped Shaft</t>
+          <t>4x Capped Shaft</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2x Pitch Capped Shaft</t>
+          <t>4x Pitch Capped Shaft</t>
         </is>
       </c>
     </row>
@@ -3130,12 +3126,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>3x Capped Shaft</t>
+          <t>5x Capped Shafts (metal + plastic)</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>3x Pitch Capped Shaft</t>
+          <t>5x Pitch Capped Plastic Shaft</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>5x Pitch Capped Shaft</t>
         </is>
       </c>
     </row>
@@ -3152,12 +3153,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4x Capped Shaft</t>
+          <t>1x Plastic Motor Shaft</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>4x Pitch Capped Shaft</t>
+          <t>1x Pitch Plastic Motor Shaft</t>
         </is>
       </c>
     </row>
@@ -3174,12 +3175,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>5x Capped Shaft</t>
+          <t>2x Motor Shafts (plastic + metal)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>5x Pitch Capped Shaft</t>
+          <t>2x Pitch Plastic Motor Shaft</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2x Pitch Motor Shaft</t>
         </is>
       </c>
     </row>
@@ -3196,12 +3202,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2x Motor Shaft</t>
+          <t>3x Motor Shafts (plastic + metal)</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2x Pitch Motor Shaft</t>
+          <t>3x Pitch Plastic Motor Shaft</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>3x Pitch Motor Shaft</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3229,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>3x Motor Shaft</t>
+          <t>4x Motor Shafts (plastic + metal)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>3x Pitch Motor Shaft</t>
+          <t>4x Pitch Plastic Motor Shaft</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>4x Pitch Motor Shaft</t>
         </is>
       </c>
     </row>
@@ -3238,16 +3254,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>4x Motor Shaft</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>4x Pitch Motor Shaft</t>
-        </is>
-      </c>
+      <c r="C120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
@@ -3306,12 +3313,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1x1 Idler Pin</t>
+          <t>0x2 Idler Pin</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>1x1 Idler Pin</t>
+          <t>0x2 Idler Pin</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3335,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>0x2 Idler Pin</t>
+          <t>0x3 Idler Pin</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>0x2 Idler Pin</t>
+          <t>0x3 Idler Pin</t>
         </is>
       </c>
     </row>
@@ -3350,12 +3357,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>0x3 Idler Pin</t>
+          <t>1x1 Idler Pin</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0x3 Idler Pin</t>
+          <t>1x1 Idler Pin</t>
         </is>
       </c>
     </row>
@@ -3392,16 +3399,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>0.25x Spacer</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>0.25x Pitch Spacer</t>
-        </is>
-      </c>
+      <c r="C127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
@@ -3416,12 +3414,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>0.5x Spacer</t>
+          <t>0.25x Standoff</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>0.5x Pitch Spacer</t>
+          <t>0.25x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3438,12 +3436,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Shaft Bushing</t>
+          <t>0.5x Standoff</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Shaft Bushing</t>
+          <t>0.5x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3460,12 +3458,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>0.25x Standoff</t>
+          <t>1x Standoff</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>0.25x Pitch Standoff</t>
+          <t>1x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3480,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>0.5x Standoff</t>
+          <t>2x Standoff</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>0.5x Pitch Standoff</t>
+          <t>2x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3504,12 +3502,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>1x Standoff</t>
+          <t>2x Standoff</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>1x Pitch Standoff</t>
+          <t>2x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3526,12 +3524,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2x Standoff</t>
+          <t>4x Standoff</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2x Pitch Standoff</t>
+          <t>4x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3548,12 +3546,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>4x Standoff</t>
+          <t>6x Standoff</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>4x Pitch Standoff</t>
+          <t>6x Pitch Standoff</t>
         </is>
       </c>
     </row>
@@ -3590,16 +3588,7 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>0.5x Standoff Extender</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>0.5x Pitch Standoff Extender</t>
-        </is>
-      </c>
+      <c r="C136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
@@ -3612,7 +3601,16 @@
           <t>Akro-Mils</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>0.5x Standoff Extender</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>0.5x Pitch Standoff Extender</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
@@ -4250,7 +4248,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="D2:H179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not a known part" error="Pick a part name from the suggestions (see the Parts tab)." type="list">
-      <formula1>=Parts!$A$2:$A$164</formula1>
+      <formula1>=Parts!$A$2:$A$163</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4263,7 +4261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5678,12 +5676,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Elastic Band Anchor Plate</t>
+          <t>Rubber Band Anchor</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Beams &amp; Plates</t>
+          <t>Specialty</t>
         </is>
       </c>
       <c r="C57" s="10">
@@ -5696,14 +5694,14 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>228-3616-157</t>
+          <t>228-2500-157, 228-3616-157</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Rubber Band Anchor</t>
+          <t>Silicone Rubber Band #32</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5721,19 +5719,19 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>228-2500-157</t>
+          <t>228-2500-468</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Silicone Rubber Band #32</t>
+          <t>North Pole Magnetic Beam</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Specialty</t>
+          <t>Beams &amp; Plates</t>
         </is>
       </c>
       <c r="C59" s="10">
@@ -5746,14 +5744,14 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>228-2500-468</t>
+          <t>228-3167-020</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>North Pole Magnetic Beam</t>
+          <t>South Pole Magnetic Beam</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5771,14 +5769,14 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>228-3167-020</t>
+          <t>228-3167-010</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>South Pole Magnetic Beam</t>
+          <t>1x12 Beam</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5796,14 +5794,14 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>228-3167-010</t>
+          <t>228-2500-011, 228-3616-011</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1x12 Beam</t>
+          <t>2x12 Beam</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5821,14 +5819,14 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>228-2500-011, 228-3616-011</t>
+          <t>228-2500-026, 228-3616-026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2x12 Beam</t>
+          <t>1x16 Beam</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5846,14 +5844,14 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>228-2500-026, 228-3616-026</t>
+          <t>228-2500-014</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1x16 Beam</t>
+          <t>2x16 Beam</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5871,14 +5869,14 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>228-2500-014</t>
+          <t>228-2500-028, 228-3616-028</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2x16 Beam</t>
+          <t>3x3 Plate</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5896,14 +5894,14 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>228-2500-028, 228-3616-028</t>
+          <t>228-2500-031</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>3x3 Plate</t>
+          <t>4x4 Plate</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -5921,14 +5919,14 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>228-2500-031</t>
+          <t>228-2500-040, 228-3616-040</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4x4 Plate</t>
+          <t>4x12 Plate</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5946,14 +5944,14 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>228-2500-040, 228-3616-040</t>
+          <t>228-3616-045</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>4x12 Plate</t>
+          <t>4x8 Plate</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -5971,19 +5969,19 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>228-3616-045</t>
+          <t>228-2500-043</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>4x8 Plate</t>
+          <t>Chain Link</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Beams &amp; Plates</t>
+          <t>Sprockets &amp; Chain</t>
         </is>
       </c>
       <c r="C69" s="10">
@@ -5996,19 +5994,19 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>228-2500-043</t>
+          <t>228-2500-230, 228-3616-230</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Chain Link</t>
+          <t>XL Turntable 36 Tooth Ring Gear Bushing</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Sprockets &amp; Chain</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C70" s="10">
@@ -6021,19 +6019,19 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>228-2500-230, 228-3616-230</t>
+          <t>228-3944-202</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>XL Turntable 36 Tooth Ring Gear Bushing</t>
+          <t>XL Turntable Outer Housing</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Specialty</t>
         </is>
       </c>
       <c r="C71" s="10">
@@ -6046,19 +6044,19 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>228-3944-202</t>
+          <t>228-3616-199</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>XL Turntable Outer Housing</t>
+          <t>XL Turntable Plain Bushing</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Specialty</t>
+          <t>Shafts &amp; Rotation</t>
         </is>
       </c>
       <c r="C72" s="10">
@@ -6071,19 +6069,19 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>228-3616-199</t>
+          <t>228-3944-200</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>XL Turntable Plain Bushing</t>
+          <t>Small Wheel Hub (44mm)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Shafts &amp; Rotation</t>
+          <t>Wheels &amp; Intake</t>
         </is>
       </c>
       <c r="C73" s="10">
@@ -6096,14 +6094,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>228-3944-200</t>
+          <t>228-2500-1208</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Small Wheel Hub (44mm)</t>
+          <t>Tire (200 mm Travel)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6121,14 +6119,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>228-2500-1208</t>
+          <t>228-2500-209</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tire (200 mm Travel)</t>
+          <t>2x Wide, 5x Pitch Diameter Balloon Tire (Racing Slick Tread)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -6146,14 +6144,14 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>228-2500-209</t>
+          <t>228-2500-1958</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2x Wide, 5x Pitch Diameter Balloon Tire (Racing Slick Tread)</t>
+          <t>2x Wide, Ø48.5mm Diameter Hub</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6171,14 +6169,14 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>228-2500-1958</t>
+          <t>228-2500-1953</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2x Wide, Ø48.5mm Diameter Hub</t>
+          <t>Omni Wheels</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6196,19 +6194,19 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>228-2500-1953</t>
+          <t>228-2536-000</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Omni Wheels</t>
+          <t>Linear Slide Bracket</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Wheels &amp; Intake</t>
+          <t>Specialty</t>
         </is>
       </c>
       <c r="C78" s="10">
@@ -6221,19 +6219,19 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>228-2536-000</t>
+          <t>228-3196-217</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Linear Slide Bracket</t>
+          <t>Rack Gear</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Specialty</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C79" s="10">
@@ -6246,19 +6244,19 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>228-3196-217</t>
+          <t>228-3196-216</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Rack Gear</t>
+          <t>1x1 Beam</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Beams &amp; Plates</t>
         </is>
       </c>
       <c r="C80" s="10">
@@ -6271,14 +6269,14 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>228-3196-216</t>
+          <t>228-2500-154</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1x1 Beam</t>
+          <t>1x3 Beam</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -6296,14 +6294,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>228-2500-154</t>
+          <t>228-3616-002</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1x3 Beam</t>
+          <t>1x5 Beam</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6321,14 +6319,14 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>228-3616-002</t>
+          <t>228-2500-004</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1x5 Beam</t>
+          <t>1x3 Center Lock Beam</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6346,14 +6344,14 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>228-2500-004</t>
+          <t>228-2500-1141</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1x3 Center Lock Beam</t>
+          <t>1x3 Center Lock Plate</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6371,14 +6369,14 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>228-2500-1141</t>
+          <t>228-3201-141</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1x3 Center Lock Plate</t>
+          <t>1x4 Low-Profile End Lock Beam</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6396,14 +6394,14 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>228-3201-141</t>
+          <t>228-2500-1548</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1x4 Low-Profile End Lock Beam</t>
+          <t>2x2 Center Offset Round Lock Beam</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -6421,14 +6419,14 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>228-2500-1548</t>
+          <t>228-2500-1925</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2x2 Center Offset Round Lock Beam</t>
+          <t>2x2 Lock Plate</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6446,19 +6444,19 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>228-2500-1925</t>
+          <t>228-3201-140</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2x2 Lock Plate</t>
+          <t>12 Tooth Gear</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Beams &amp; Plates</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C88" s="10">
@@ -6471,14 +6469,14 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>228-3201-140</t>
+          <t>228-2500-213, 228-3196-213</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>12 Tooth Gear</t>
+          <t>24 Tooth Gear</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6496,14 +6494,14 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>228-2500-213, 228-3196-213</t>
+          <t>228-2500-227</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>24 Tooth Gear</t>
+          <t>36 Tooth Gear</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6521,14 +6519,14 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>228-2500-227</t>
+          <t>228-2500-214, 228-3196-214</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>36 Tooth Gear</t>
+          <t>48 Tooth Gear</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6546,14 +6544,14 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>228-2500-214, 228-3196-214</t>
+          <t>228-2500-228</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>48 Tooth Gear</t>
+          <t>60 Tooth Gear</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6571,14 +6569,14 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>228-2500-228</t>
+          <t>228-3196-215</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>60 Tooth Gear</t>
+          <t>36 Tooth Crown Gear</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -6596,14 +6594,14 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>228-3196-215</t>
+          <t>228-3196-218</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>36 Tooth Crown Gear</t>
+          <t>Worm Bracket</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -6621,14 +6619,14 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>228-3196-218</t>
+          <t>228-3196-220</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Worm Bracket</t>
+          <t>Worm Gear</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -6646,14 +6644,14 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>228-3196-220</t>
+          <t>228-3196-219</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Worm Gear</t>
+          <t>1x4 Crank Arm with 23 Tooth Gear</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -6671,19 +6669,19 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>228-3196-219</t>
+          <t>228-2500-246</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1x4 Crank Arm with 23 Tooth Gear</t>
+          <t>8 Tooth Sprocket</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Sprockets &amp; Chain</t>
         </is>
       </c>
       <c r="C97" s="10">
@@ -6696,14 +6694,14 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>228-2500-246</t>
+          <t>228-2500-232, 228-3450-232</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>8 Tooth Sprocket</t>
+          <t>16 Tooth Sprocket</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6721,14 +6719,14 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>228-2500-232, 228-3450-232</t>
+          <t>228-2500-233, 228-3450-233</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>16 Tooth Sprocket</t>
+          <t>24 Tooth Sprocket</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -6746,14 +6744,14 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>228-2500-233, 228-3450-233</t>
+          <t>228-2500-235, 228-3450-235</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>24 Tooth Sprocket</t>
+          <t>32 Tooth Sprocket</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6771,14 +6769,14 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>228-2500-235, 228-3450-235</t>
+          <t>228-3450-236</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>32 Tooth Sprocket</t>
+          <t>40 Tooth Sprocket</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6796,19 +6794,19 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>228-3450-236</t>
+          <t>228-3450-237</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>40 Tooth Sprocket</t>
+          <t>10mm Pulley</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sprockets &amp; Chain</t>
+          <t>Pulleys &amp; Belts</t>
         </is>
       </c>
       <c r="C102" s="10">
@@ -6821,14 +6819,14 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>228-3450-237</t>
+          <t>228-3196-163</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>10mm Pulley</t>
+          <t>20mm Pulley</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6846,14 +6844,14 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>228-3196-163</t>
+          <t>228-3196-164</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>20mm Pulley</t>
+          <t>20mm Pulley Tire Add-On</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6871,14 +6869,14 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>228-3196-164</t>
+          <t>228-3447-207</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>20mm Pulley Tire Add-On</t>
+          <t>30mm Pulley</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6896,14 +6894,14 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>228-3447-207</t>
+          <t>228-3196-165</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>30mm Pulley</t>
+          <t>40mm Pulley</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6921,14 +6919,14 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>228-3196-165</t>
+          <t>228-3196-166</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>40mm Pulley</t>
+          <t>Belt (2mm thick x 30mm dia)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6946,14 +6944,14 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>228-3196-166</t>
+          <t>228-3447-221</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Belt (2mm thick x 30mm dia)</t>
+          <t>Belt (2mm thick x 40mm dia)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6971,14 +6969,14 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>228-3447-221</t>
+          <t>228-3447-222</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Belt (2mm thick x 40mm dia)</t>
+          <t>Belt (2mm thick x 50mm dia)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6996,14 +6994,14 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>228-3447-222</t>
+          <t>228-3447-223</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Belt (2mm thick x 50mm dia)</t>
+          <t>Belt (2mm thick x 60mm dia)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -7021,19 +7019,19 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>228-3447-223</t>
+          <t>228-3447-224</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Belt (2mm thick x 60mm dia)</t>
+          <t>1x Pitch Plastic Motor Shaft</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Pulleys &amp; Belts</t>
+          <t>Shafts &amp; Rotation</t>
         </is>
       </c>
       <c r="C111" s="10">
@@ -7046,14 +7044,14 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>228-3447-224</t>
+          <t>228-2500-328</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>1x Pitch Plastic Motor Shaft</t>
+          <t>2x Pitch Plastic Motor Shaft</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -7071,14 +7069,14 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>228-2500-328</t>
+          <t>228-2500-078</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2x Pitch Plastic Motor Shaft</t>
+          <t>3x Pitch Plastic Motor Shaft</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -7096,14 +7094,14 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>228-2500-078</t>
+          <t>228-2500-094</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>3x Pitch Plastic Motor Shaft</t>
+          <t>4x Pitch Plastic Motor Shaft</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -7121,14 +7119,14 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>228-2500-094</t>
+          <t>228-2500-079</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>4x Pitch Plastic Motor Shaft</t>
+          <t>3x Pitch Capped Plastic Shaft</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -7146,14 +7144,14 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>228-2500-079</t>
+          <t>228-2500-081</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>3x Pitch Capped Plastic Shaft</t>
+          <t>5x Pitch Capped Plastic Shaft</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -7171,14 +7169,14 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>228-2500-081</t>
+          <t>228-2500-083</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>5x Pitch Capped Plastic Shaft</t>
+          <t>2x Pitch Capped Shaft</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -7196,14 +7194,14 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>228-2500-083</t>
+          <t>228-2500-2219</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2x Pitch Capped Shaft</t>
+          <t>3x Pitch Capped Shaft</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -7221,14 +7219,14 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>228-2500-2219</t>
+          <t>228-2500-2221</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>3x Pitch Capped Shaft</t>
+          <t>4x Pitch Capped Shaft</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7246,14 +7244,14 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>228-2500-2221</t>
+          <t>228-2500-2223</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>4x Pitch Capped Shaft</t>
+          <t>5x Pitch Capped Shaft</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7271,14 +7269,14 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>228-2500-2223</t>
+          <t>228-2500-2225</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>5x Pitch Capped Shaft</t>
+          <t>2x Pitch Motor Shaft</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7296,14 +7294,14 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>228-2500-2225</t>
+          <t>228-2500-2234</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2x Pitch Motor Shaft</t>
+          <t>3x Pitch Motor Shaft</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7321,14 +7319,14 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>228-2500-2234</t>
+          <t>228-2500-2236</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>3x Pitch Motor Shaft</t>
+          <t>4x Pitch Motor Shaft</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7346,19 +7344,19 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>228-2500-2236</t>
+          <t>228-2500-2238</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>4x Pitch Motor Shaft</t>
+          <t>0x2 Connector Pin</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Shafts &amp; Rotation</t>
+          <t>Pins &amp; Standoffs</t>
         </is>
       </c>
       <c r="C124" s="10">
@@ -7371,14 +7369,14 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>228-2500-2238</t>
+          <t>228-2500-086</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>0x2 Connector Pin</t>
+          <t>0x3 Connector Pin</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7396,14 +7394,14 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>228-2500-086</t>
+          <t>228-2500-087</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>0x3 Connector Pin</t>
+          <t>1x1 Idler Pin</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7421,14 +7419,14 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>228-2500-087</t>
+          <t>228-2500-073</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>1x1 Idler Pin</t>
+          <t>0x2 Idler Pin</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7446,14 +7444,14 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>228-2500-073</t>
+          <t>228-2500-084, 228-3944-084</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>0x2 Idler Pin</t>
+          <t>0x3 Idler Pin</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7471,14 +7469,14 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>228-2500-084, 228-3944-084</t>
+          <t>228-3944-097</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>0x3 Idler Pin</t>
+          <t>1x2 Idler Pin</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7496,19 +7494,19 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>228-3944-097</t>
+          <t>228-3944-098</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>1x2 Idler Pin</t>
+          <t>0.25x Pitch Spacer</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Pins &amp; Standoffs</t>
+          <t>Shafts &amp; Rotation</t>
         </is>
       </c>
       <c r="C130" s="10">
@@ -7521,14 +7519,14 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>228-3944-098</t>
+          <t>228-2500-114</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>0.25x Pitch Spacer</t>
+          <t>0.5x Pitch Spacer</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7546,14 +7544,14 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>228-2500-114</t>
+          <t>228-3201-114</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>0.5x Pitch Spacer</t>
+          <t>Shaft Bushing</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7571,19 +7569,19 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>228-3201-114</t>
+          <t>228-3201-125</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Shaft Bushing</t>
+          <t>0.25x Pitch Standoff</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Shafts &amp; Rotation</t>
+          <t>Pins &amp; Standoffs</t>
         </is>
       </c>
       <c r="C133" s="10">
@@ -7596,14 +7594,14 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>228-3201-125</t>
+          <t>228-2500-063</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>0.25x Pitch Standoff</t>
+          <t>0.5x Pitch Standoff</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7621,14 +7619,14 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>228-2500-063</t>
+          <t>228-2500-064, 228-3201-064</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>0.5x Pitch Standoff</t>
+          <t>1x Pitch Standoff</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7646,14 +7644,14 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>228-2500-064, 228-3201-064</t>
+          <t>228-2500-065, 228-3201-065</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>1x Pitch Standoff</t>
+          <t>2x Pitch Standoff</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7671,14 +7669,14 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>228-2500-065, 228-3201-065</t>
+          <t>228-2500-067, 228-3201-067</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2x Pitch Standoff</t>
+          <t>4x Pitch Standoff</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7696,14 +7694,14 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>228-2500-067, 228-3201-067</t>
+          <t>228-2500-070, 228-3201-070</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>4x Pitch Standoff</t>
+          <t>6x Pitch Standoff</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7721,14 +7719,14 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>228-2500-070, 228-3201-070</t>
+          <t>228-2500-072, 228-3201-072</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>6x Pitch Standoff</t>
+          <t>0.5x Pitch Standoff Extender</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -7746,19 +7744,19 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>228-2500-072, 228-3201-072</t>
+          <t>228-2500-109</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>0.5x Pitch Standoff Extender</t>
+          <t>2x18 Beam</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Pins &amp; Standoffs</t>
+          <t>Beams &amp; Plates</t>
         </is>
       </c>
       <c r="C140" s="10">
@@ -7771,14 +7769,14 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>228-2500-109</t>
+          <t>228-2500-029</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2x18 Beam</t>
+          <t>2x20 Beam</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -7796,19 +7794,19 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>228-2500-029</t>
+          <t>228-2500-030, 228-3616-030</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2x20 Beam</t>
+          <t>200mm Cable</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Beams &amp; Plates</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C142" s="10">
@@ -7821,14 +7819,14 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>228-2500-030, 228-3616-030</t>
+          <t>228-2780-001</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>200mm Cable</t>
+          <t>300mm Cable</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -7846,14 +7844,14 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>228-2780-001</t>
+          <t>228-2780-002</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>300mm Cable</t>
+          <t>400mm Cable</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -7871,14 +7869,14 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>228-2780-002</t>
+          <t>228-2780-003</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>400mm Cable</t>
+          <t>600mm Cable</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -7896,14 +7894,14 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>228-2780-003</t>
+          <t>228-2780-004</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>600mm Cable</t>
+          <t>USB A-C Cable</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -7921,19 +7919,19 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>228-2780-004</t>
+          <t>228-6961-002</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>USB A-C Cable</t>
+          <t>Robot Brain (2nd generation)</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="C147" s="10">
@@ -7946,14 +7944,14 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>228-6961-002</t>
+          <t>228-6480-000</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Robot Brain (2nd generation)</t>
+          <t>Controller (2nd Generation)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7971,14 +7969,14 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>228-6480-000</t>
+          <t>228-6470-000</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Controller (2nd Generation)</t>
+          <t>Robot Battery (Li-Ion, 2000 mAh)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -7996,14 +7994,14 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>228-6470-000</t>
+          <t>228-7045-000</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Robot Battery (Li-Ion, 2000 mAh)</t>
+          <t>Smart Motor</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -8021,19 +8019,19 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>228-7045-000</t>
+          <t>228-2560-000</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Smart Motor</t>
+          <t>Bumper Switch</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="C151" s="10">
@@ -8046,14 +8044,14 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>228-2560-000</t>
+          <t>228-2677-000</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Bumper Switch</t>
+          <t>Distance Sensor</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -8071,14 +8069,14 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>228-2677-000</t>
+          <t>228-7106-000</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Distance Sensor</t>
+          <t>Optical Sensor</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -8096,14 +8094,14 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>228-7106-000</t>
+          <t>228-7082-000</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Optical Sensor</t>
+          <t>Touch LED</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -8121,19 +8119,19 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>228-7082-000</t>
+          <t>228-3010-000</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Touch LED</t>
+          <t>Pin Tool</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Pins &amp; Standoffs</t>
         </is>
       </c>
       <c r="C155" s="10">
@@ -8146,19 +8144,19 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>228-3010-000</t>
+          <t>228-4035-000</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Pin Tool</t>
+          <t>1x5 Linear Motion Beam</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Pins &amp; Standoffs</t>
+          <t>Linear Motion</t>
         </is>
       </c>
       <c r="C156" s="10">
@@ -8171,14 +8169,14 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>228-4035-000</t>
+          <t>228-2500-1456</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>1x5 Linear Motion Beam</t>
+          <t>1x6 Linear Motion Beam</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -8196,14 +8194,14 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>228-2500-1456</t>
+          <t>228-2500-1457</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>1x6 Linear Motion Beam</t>
+          <t>1x8 Linear Motion Beam</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -8221,14 +8219,14 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>228-2500-1457</t>
+          <t>228-2500-1459</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>1x8 Linear Motion Beam</t>
+          <t>1x6 Linear Motion Rack Gear</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -8246,14 +8244,14 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>228-2500-1459</t>
+          <t>228-2500-1472</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>1x6 Linear Motion Rack Gear</t>
+          <t>1x6 Continuous Linear Motion Rack Gear</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -8271,14 +8269,14 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>228-2500-1472</t>
+          <t>228-2500-1473</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>1x6 Continuous Linear Motion Rack Gear</t>
+          <t>1x20 Linear Motion Rack Gear</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -8296,14 +8294,14 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>228-2500-1473</t>
+          <t>228-2500-1454</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>1x20 Linear Motion Rack Gear</t>
+          <t>2x Pitch Linear Motion Bracket (Side Mount)</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -8321,14 +8319,14 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>228-2500-1454</t>
+          <t>228-2500-1469</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2x Pitch Linear Motion Bracket (Side Mount)</t>
+          <t>1x Pitch Linear Motion Bracket (Snap Mount)</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -8346,38 +8344,13 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>228-2500-1469</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>1x Pitch Linear Motion Bracket (Snap Mount)</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Linear Motion</t>
-        </is>
-      </c>
-      <c r="C164" s="10">
-        <f t="array" ref="C164">TEXTJOIN(", ",TRUE,IF((Bins!$D$2:$D$179=A164)+(Bins!$E$2:$E$179=A164)+(Bins!$F$2:$F$179=A164)+(Bins!$G$2:$G$179=A164)+(Bins!$H$2:$H$179=A164),Bins!$A$2:$A$179,""))</f>
-        <v/>
-      </c>
-      <c r="D164" s="10">
-        <f>COUNTIF(Bins!$D$2:$H$179,A164)</f>
-        <v/>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
           <t>228-2500-1470</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E164"/>
-  <conditionalFormatting sqref="D2:D164">
+  <autoFilter ref="A1:E163"/>
+  <conditionalFormatting sqref="D2:D163">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>D2=0</formula>
     </cfRule>

</xml_diff>